<commit_message>
create and test month acts generate for all houses and one
</commit_message>
<xml_diff>
--- a/back-end/mkd_works_service/api/templates/year_act/mkd_services_year_act_template_v2.xlsx
+++ b/back-end/mkd_works_service/api/templates/year_act/mkd_services_year_act_template_v2.xlsx
@@ -8,13 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Projects\Housing Company Services(HCS)\back-end\mkd_works_service\api\templates\year_act\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{814E0135-C27A-4E18-A275-CBEDABEB46E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43029141-F450-46BD-A5FC-2E5F5EB15499}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6420" yWindow="3225" windowWidth="21600" windowHeight="11385" xr2:uid="{45563469-E7B0-4AAB-8A11-B677FF13F0C3}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{45563469-E7B0-4AAB-8A11-B677FF13F0C3}"/>
   </bookViews>
   <sheets>
     <sheet name="Лист1" sheetId="1" r:id="rId1"/>
-    <sheet name="Лист2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -35,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="27">
   <si>
     <t>УТВЕРЖДЕНО приказом Министерства строительства и жилищно- коммунального хозяйства Российской Федерации от 26.10.2015 N 761/пр</t>
   </si>
@@ -114,33 +113,6 @@
   </si>
   <si>
     <t>Цена выполненной работы (оказанной услуги), в рублях</t>
-  </si>
-  <si>
-    <t xml:space="preserve">         2. Всего за период с {{ start_work_date }} по {{ end_work_date }} выполнено работ (оказано услуг) на общую сумму</t>
-  </si>
-  <si>
-    <t xml:space="preserve">        {{ all_work_sum }} руб.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">         3. Работы (услуги) выполнены (оказаны) полностью, в установленные сроки, с надлежащим качеством. </t>
-  </si>
-  <si>
-    <t xml:space="preserve">         4. Претензий по выполнению условий Договора Стороны друг к другу не имеют. Настоящий Акт составлен в</t>
-  </si>
-  <si>
-    <t xml:space="preserve">       2 экземплярах, имеющих одинаковую юридическую силу, по одному для каждой из Сторон</t>
-  </si>
-  <si>
-    <t>Подписи Сторон:</t>
-  </si>
-  <si>
-    <t>Исполнитель -              Генеральный директор  {{company_director}}</t>
-  </si>
-  <si>
-    <t>(подпись)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Заказчик -                     </t>
   </si>
   <si>
     <t xml:space="preserve">       №   ______   от "                                                                          "                      г. (далее - "Договор") услуги и (или)</t>
@@ -230,7 +202,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -246,20 +218,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -267,7 +231,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
@@ -605,31 +568,31 @@
       </c>
     </row>
     <row r="2" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A2" s="12" t="s">
+      <c r="A2" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="12"/>
-      <c r="C2" s="12"/>
-      <c r="D2" s="12"/>
-      <c r="E2" s="12"/>
+      <c r="B2" s="10"/>
+      <c r="C2" s="10"/>
+      <c r="D2" s="10"/>
+      <c r="E2" s="10"/>
     </row>
     <row r="3" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A3" s="13" t="s">
+      <c r="A3" s="11" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="13"/>
-      <c r="C3" s="13"/>
-      <c r="D3" s="13"/>
-      <c r="E3" s="13"/>
+      <c r="B3" s="11"/>
+      <c r="C3" s="11"/>
+      <c r="D3" s="11"/>
+      <c r="E3" s="11"/>
     </row>
     <row r="4" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A4" s="13" t="s">
+      <c r="A4" s="11" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="13"/>
-      <c r="C4" s="13"/>
-      <c r="D4" s="13"/>
-      <c r="E4" s="13"/>
+      <c r="B4" s="11"/>
+      <c r="C4" s="11"/>
+      <c r="D4" s="11"/>
+      <c r="E4" s="11"/>
     </row>
     <row r="5" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A5" s="3"/>
@@ -729,7 +692,7 @@
       <c r="E15" s="9"/>
     </row>
     <row r="16" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A16" s="11" t="s">
+      <c r="A16" s="8" t="s">
         <v>14</v>
       </c>
       <c r="B16" s="9"/>
@@ -775,7 +738,7 @@
     </row>
     <row r="21" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A21" s="9" t="s">
-        <v>35</v>
+        <v>26</v>
       </c>
       <c r="B21" s="9"/>
       <c r="C21" s="9"/>
@@ -825,14 +788,21 @@
       </c>
     </row>
     <row r="26" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A26" s="14"/>
-      <c r="B26" s="14"/>
-      <c r="C26" s="14"/>
-      <c r="D26" s="14"/>
-      <c r="E26" s="14"/>
+      <c r="A26" s="7"/>
+      <c r="B26" s="7"/>
+      <c r="C26" s="7"/>
+      <c r="D26" s="7"/>
+      <c r="E26" s="7"/>
     </row>
   </sheetData>
   <mergeCells count="19">
+    <mergeCell ref="A22:E22"/>
+    <mergeCell ref="A23:E23"/>
+    <mergeCell ref="A17:E17"/>
+    <mergeCell ref="A18:E18"/>
+    <mergeCell ref="A19:E19"/>
+    <mergeCell ref="A20:E20"/>
+    <mergeCell ref="A21:E21"/>
     <mergeCell ref="A16:E16"/>
     <mergeCell ref="A2:E2"/>
     <mergeCell ref="A3:E3"/>
@@ -845,151 +815,8 @@
     <mergeCell ref="A13:E13"/>
     <mergeCell ref="A14:E14"/>
     <mergeCell ref="A15:E15"/>
-    <mergeCell ref="A17:E17"/>
-    <mergeCell ref="A18:E18"/>
-    <mergeCell ref="A19:E19"/>
-    <mergeCell ref="A20:E20"/>
-    <mergeCell ref="A21:E21"/>
-    <mergeCell ref="A22:E22"/>
-    <mergeCell ref="A23:E23"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="77" fitToHeight="0" orientation="portrait" r:id="rId1"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8EEF2203-E962-465B-8B8A-8FD7CF2BA0B6}">
-  <dimension ref="A1:E14"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="22.42578125" customWidth="1"/>
-    <col min="2" max="2" width="17.42578125" customWidth="1"/>
-    <col min="3" max="3" width="19.7109375" customWidth="1"/>
-    <col min="4" max="4" width="20.85546875" customWidth="1"/>
-    <col min="5" max="5" width="37.42578125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A1" s="1"/>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-    </row>
-    <row r="2" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A2" s="8" t="s">
-        <v>26</v>
-      </c>
-      <c r="B2" s="8"/>
-      <c r="C2" s="8"/>
-      <c r="D2" s="8"/>
-      <c r="E2" s="8"/>
-    </row>
-    <row r="3" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="B3" s="1"/>
-      <c r="C3" s="1"/>
-      <c r="D3" s="1"/>
-      <c r="E3" s="1"/>
-    </row>
-    <row r="4" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A4" s="10" t="s">
-        <v>28</v>
-      </c>
-      <c r="B4" s="10"/>
-      <c r="C4" s="10"/>
-      <c r="D4" s="10"/>
-      <c r="E4" s="10"/>
-    </row>
-    <row r="5" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A5" s="8" t="s">
-        <v>29</v>
-      </c>
-      <c r="B5" s="8"/>
-      <c r="C5" s="8"/>
-      <c r="D5" s="8"/>
-      <c r="E5" s="8"/>
-    </row>
-    <row r="6" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A6" s="9" t="s">
-        <v>30</v>
-      </c>
-      <c r="B6" s="9"/>
-      <c r="C6" s="9"/>
-      <c r="D6" s="9"/>
-      <c r="E6" s="9"/>
-    </row>
-    <row r="7" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A7" s="1"/>
-      <c r="B7" s="1"/>
-      <c r="C7" s="1"/>
-      <c r="D7" s="1"/>
-      <c r="E7" s="1"/>
-    </row>
-    <row r="8" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A8" s="7" t="s">
-        <v>31</v>
-      </c>
-      <c r="B8" s="7"/>
-      <c r="C8" s="7"/>
-      <c r="D8" s="7"/>
-      <c r="E8" s="7"/>
-    </row>
-    <row r="9" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A9" s="1"/>
-      <c r="B9" s="1"/>
-      <c r="C9" s="1"/>
-      <c r="D9" s="1"/>
-      <c r="E9" s="1"/>
-    </row>
-    <row r="10" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A10" s="8" t="s">
-        <v>32</v>
-      </c>
-      <c r="B10" s="8"/>
-      <c r="C10" s="8"/>
-      <c r="D10" s="8"/>
-      <c r="E10" s="8"/>
-    </row>
-    <row r="11" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A11" s="1"/>
-      <c r="B11" s="1"/>
-      <c r="C11" s="1"/>
-      <c r="D11" s="7" t="s">
-        <v>33</v>
-      </c>
-      <c r="E11" s="7"/>
-    </row>
-    <row r="13" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A13" s="8" t="s">
-        <v>34</v>
-      </c>
-      <c r="B13" s="8"/>
-      <c r="C13" s="8"/>
-      <c r="D13" s="8"/>
-      <c r="E13" s="8"/>
-    </row>
-    <row r="14" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="D14" s="7" t="s">
-        <v>33</v>
-      </c>
-      <c r="E14" s="7"/>
-    </row>
-  </sheetData>
-  <mergeCells count="9">
-    <mergeCell ref="D11:E11"/>
-    <mergeCell ref="A13:E13"/>
-    <mergeCell ref="D14:E14"/>
-    <mergeCell ref="A6:E6"/>
-    <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A4:E4"/>
-    <mergeCell ref="A5:E5"/>
-    <mergeCell ref="A8:E8"/>
-    <mergeCell ref="A10:E10"/>
-  </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>